<commit_message>
Completamento struttura txt_generator per la creazione dei file txt
</commit_message>
<xml_diff>
--- a/documenti/Struttura log.xlsx
+++ b/documenti/Struttura log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\Avanzamenti_produzione\documenti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6700613-CCC8-4447-8A9E-507E602B1C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2999960-3C73-48E8-8B8E-D9CE062E179C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{E8EB9653-BC78-422A-B6D5-0640D099AC7F}"/>
+    <workbookView xWindow="-28920" yWindow="1800" windowWidth="29040" windowHeight="15720" tabRatio="430" activeTab="1" xr2:uid="{E8EB9653-BC78-422A-B6D5-0640D099AC7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -391,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -399,23 +399,20 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1090,17 +1087,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="E2" s="6" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="E2" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="7"/>
       <c r="I2" s="2" t="s">
         <v>28</v>
       </c>
@@ -1154,7 +1151,7 @@
       </c>
     </row>
     <row r="3" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1163,13 +1160,13 @@
       <c r="C3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="8">
         <v>1</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="6" t="s">
         <v>67</v>
       </c>
       <c r="I3" s="2" t="s">
@@ -1198,7 +1195,7 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
+      <c r="A4" s="5">
         <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1207,13 +1204,13 @@
       <c r="C4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="8">
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="6" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -1260,7 +1257,7 @@
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="5">
         <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1269,18 +1266,18 @@
       <c r="C5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="8">
         <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="7">
+      <c r="A6" s="5">
         <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1289,19 +1286,19 @@
       <c r="C6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="8">
         <v>30</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="6" t="s">
         <v>12</v>
       </c>
       <c r="I6" s="3"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="5">
         <v>40</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1310,33 +1307,33 @@
       <c r="C7" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="8">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="5">
         <v>80</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="7">
+      <c r="C8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="5">
         <v>80</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="6">
         <v>701</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -1377,22 +1374,22 @@
       </c>
     </row>
     <row r="9" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="5">
         <v>90</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="7">
+      <c r="C9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="5">
         <v>90</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="6" t="s">
         <v>47</v>
       </c>
       <c r="I9" s="2" t="s">
@@ -1418,22 +1415,22 @@
       </c>
     </row>
     <row r="10" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+      <c r="A10" s="5">
         <v>100</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="7">
+      <c r="C10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="5">
         <v>100</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="6" t="s">
         <v>88</v>
       </c>
       <c r="I10" s="2" t="s">
@@ -1465,22 +1462,22 @@
       </c>
     </row>
     <row r="11" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
+      <c r="A11" s="5">
         <v>140</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="7">
+      <c r="C11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="5">
         <v>140</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="6" t="s">
         <v>89</v>
       </c>
       <c r="I11" s="2" t="s">
@@ -1515,22 +1512,22 @@
       </c>
     </row>
     <row r="12" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+      <c r="A12" s="5">
         <v>150</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="7">
+      <c r="C12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="5">
         <v>150</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="6" t="s">
         <v>89</v>
       </c>
       <c r="I12" s="2" t="s">
@@ -1562,336 +1559,336 @@
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
+      <c r="A13" s="5">
         <v>160</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="7">
+      <c r="C13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="5">
         <v>160</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
+      <c r="A14" s="5">
         <v>290</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="7">
+      <c r="C14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="5">
         <v>290</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="6" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="7">
+      <c r="A15" s="5">
         <v>340</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="7">
+      <c r="C15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="5">
         <v>340</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="6" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="7">
+      <c r="A16" s="5">
         <v>210</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="7">
+      <c r="C16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="5">
         <v>210</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="7">
+      <c r="A17" s="5">
         <v>300</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" s="7">
+      <c r="C17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="5">
         <v>300</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="6" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="7">
+      <c r="A18" s="5">
         <v>310</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="7">
+      <c r="C18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="5">
         <v>310</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="6" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="7">
+      <c r="A19" s="5">
         <v>322</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="7">
+      <c r="C19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="5">
         <v>322</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E22" s="10">
+      <c r="E22" s="8">
         <v>1</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="6" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E23" s="10">
+      <c r="E23" s="8">
         <v>10</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E24" s="10">
+      <c r="E24" s="8">
         <v>20</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G24" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E25" s="10">
+      <c r="E25" s="8">
         <v>30</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E26" s="10">
+      <c r="E26" s="8">
         <v>40</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E27" s="7">
+      <c r="E27" s="5">
         <v>80</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="6">
         <v>701</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E28" s="7">
+      <c r="E28" s="5">
         <v>90</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="G28" s="5" t="s">
+      <c r="G28" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E29" s="7">
+      <c r="E29" s="5">
         <v>100</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="G29" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E30" s="7">
+      <c r="E30" s="5">
         <v>140</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G30" s="8" t="s">
+      <c r="G30" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E31" s="7">
+      <c r="E31" s="5">
         <v>150</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G31" s="8" t="s">
+      <c r="G31" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E32" s="7">
+      <c r="E32" s="5">
         <v>160</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="G32" s="8" t="s">
+      <c r="G32" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="33" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E33" s="7">
+      <c r="E33" s="5">
         <v>290</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="6" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="34" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E34" s="7">
+      <c r="E34" s="5">
         <v>340</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G34" s="8" t="s">
+      <c r="G34" s="6" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="35" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E35" s="7">
+      <c r="E35" s="5">
         <v>210</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G35" s="8">
+      <c r="G35" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E36" s="7">
+      <c r="E36" s="5">
         <v>300</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G36" s="8" t="s">
+      <c r="G36" s="6" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="37" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E37" s="7">
+      <c r="E37" s="5">
         <v>310</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G37" s="8" t="s">
+      <c r="G37" s="6" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="38" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E38" s="7">
+      <c r="E38" s="5">
         <v>322</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="G38" s="6" t="s">
         <v>94</v>
       </c>
     </row>

</xml_diff>